<commit_message>
Create mitigations template with dummy data (addresses #4)
</commit_message>
<xml_diff>
--- a/data/mitigations.xlsx
+++ b/data/mitigations.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">start_node</t>
   </si>
@@ -32,10 +32,16 @@
     <t xml:space="preserve">edge</t>
   </si>
   <si>
-    <t xml:space="preserve">short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">long</t>
+    <t xml:space="preserve">short_en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">long_en</t>
+  </si>
+  <si>
+    <t xml:space="preserve">short_fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">long_fr</t>
   </si>
   <si>
     <t xml:space="preserve">Selective work</t>
@@ -62,7 +68,28 @@
     <t xml:space="preserve">Remove (hunt/relocate) predators to reduce pressure. May create problems for predator species.</t>
   </si>
   <si>
-    <t xml:space="preserve">Placeholder</t>
+    <t xml:space="preserve">Option 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 8</t>
   </si>
   <si>
     <r>
@@ -202,7 +229,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -329,10 +356,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -351,6 +379,12 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
@@ -361,140 +395,140 @@
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>88</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>88</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>7</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>13</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>14</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>48</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -518,7 +552,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Allow multiple mitigation pathways per mitigation and mitigation checks
</commit_message>
<xml_diff>
--- a/data/mitigations.xlsx
+++ b/data/mitigations.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t xml:space="preserve">start_node</t>
   </si>
@@ -68,10 +68,13 @@
     <t xml:space="preserve">Remove (hunt/relocate) predators to reduce pressure. May create problems for predator species.</t>
   </si>
   <si>
-    <t xml:space="preserve">Option 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Option 2</t>
+    <t xml:space="preserve">Add Gate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Habitat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measure 1</t>
   </si>
   <si>
     <t xml:space="preserve">Option 3</t>
@@ -356,11 +359,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -444,91 +447,124 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>4</v>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="n">
+        <v>55</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>5</v>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="n">
+        <v>204</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="n">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>6</v>
-      </c>
       <c r="D8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="n">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>7</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>13</v>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="n">
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="n">
+        <v>191</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B14" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="n">
+      <c r="D15" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B16" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="n">
+      <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>22</v>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>103</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>194</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -552,7 +588,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restyle app and add custom mitigations
</commit_message>
<xml_diff>
--- a/data/mitigations.xlsx
+++ b/data/mitigations.xlsx
@@ -44,7 +44,7 @@
     <t xml:space="preserve">long_fr</t>
   </si>
   <si>
-    <t xml:space="preserve">Selective work</t>
+    <t xml:space="preserve">Selective work </t>
   </si>
   <si>
     <t xml:space="preserve">By working selectively, avoid direct problems.</t>
@@ -242,7 +242,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>